<commit_message>
mainly verified counts for half of the plots according to final results.
</commit_message>
<xml_diff>
--- a/data/verification/metadata all/datasets_metadata_master_updated/filled tables/sample_200_ids_no_citation_v14.xlsx
+++ b/data/verification/metadata all/datasets_metadata_master_updated/filled tables/sample_200_ids_no_citation_v14.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29212"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29406"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://charitede.sharepoint.com/sites/TeamOpenDataundForschungsdatenmanagement/Shared Documents/DCC analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2323" documentId="8_{74E9A759-E3F3-4C51-AE69-BA3081BA9F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{776DD6A1-5E88-4973-B1FA-436B6ED3228C}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{40BA2668-F962-4508-B9C8-BAF501DBE206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="16800" xr2:uid="{09E8D75B-4697-4AE2-9C91-7FB731FFD36E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2398" uniqueCount="601">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2411" uniqueCount="603">
   <si>
     <t>unique_id</t>
   </si>
@@ -1842,6 +1842,12 @@
   </si>
   <si>
     <t>gse148720</t>
+  </si>
+  <si>
+    <t>10.1038/s41590-023-01517-x</t>
+  </si>
+  <si>
+    <t>gse171690</t>
   </si>
 </sst>
 </file>
@@ -2729,7 +2735,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FF1161B-FCE9-4460-9050-37E197CDE322}">
-  <dimension ref="A1:T201"/>
+  <dimension ref="A1:T202"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="33.85546875" customWidth="1"/>
@@ -13562,6 +13568,62 @@
         <v>0</v>
       </c>
       <c r="S201">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="202" spans="1:20">
+      <c r="B202" t="s">
+        <v>601</v>
+      </c>
+      <c r="C202" t="s">
+        <v>601</v>
+      </c>
+      <c r="D202" t="s">
+        <v>602</v>
+      </c>
+      <c r="E202" t="s">
+        <v>602</v>
+      </c>
+      <c r="F202" t="s">
+        <v>90</v>
+      </c>
+      <c r="G202" t="s">
+        <v>91</v>
+      </c>
+      <c r="H202" t="s">
+        <v>92</v>
+      </c>
+      <c r="I202" t="s">
+        <v>91</v>
+      </c>
+      <c r="J202" t="s">
+        <v>91</v>
+      </c>
+      <c r="K202" t="s">
+        <v>98</v>
+      </c>
+      <c r="L202" t="s">
+        <v>94</v>
+      </c>
+      <c r="M202" t="s">
+        <v>99</v>
+      </c>
+      <c r="N202">
+        <v>2023</v>
+      </c>
+      <c r="O202" t="s">
+        <v>94</v>
+      </c>
+      <c r="P202">
+        <v>1</v>
+      </c>
+      <c r="Q202">
+        <v>1</v>
+      </c>
+      <c r="R202">
+        <v>1</v>
+      </c>
+      <c r="S202">
         <v>0</v>
       </c>
     </row>
@@ -13728,9 +13790,30 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100029FD0B41DD07841BED16965712E158C" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e0f1011f30fef6dde8223745cec2fc96">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="aaacefca-f467-416c-abd0-2b181dff1e20" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4d5cb4cdee1db726a521ed27371901b5" ns2:_="">
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a0e84d40-090a-490d-8a02-2942ffba970a" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="aaacefca-f467-416c-abd0-2b181dff1e20">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100029FD0B41DD07841BED16965712E158C" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ae6d51e96c8c66a8de8dfe8311f95192">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="aaacefca-f467-416c-abd0-2b181dff1e20" xmlns:ns3="a0e84d40-090a-490d-8a02-2942ffba970a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f9e171e4f7fb14517da8847a2c60885" ns2:_="" ns3:_="">
     <xsd:import namespace="aaacefca-f467-416c-abd0-2b181dff1e20"/>
+    <xsd:import namespace="a0e84d40-090a-490d-8a02-2942ffba970a"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -13741,6 +13824,12 @@
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -13770,6 +13859,50 @@
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="12" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="14" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="2375ea7b-1eef-4e91-915e-32e4cb5a9c34" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="a0e84d40-090a-490d-8a02-2942ffba970a" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="15" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b1b93042-dae5-4a91-aee7-e8b26f1570c8}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="a0e84d40-090a-490d-8a02-2942ffba970a">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
@@ -13871,29 +14004,14 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{258E5007-F839-47E8-8DD0-6390E45E526A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FBF8ED2E-F592-4203-B976-1A1E5F1160CA}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FBF8ED2E-F592-4203-B976-1A1E5F1160CA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ECD72CA5-154B-4C15-83BC-C172B74CF1C7}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ECD72CA5-154B-4C15-83BC-C172B74CF1C7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DCCFFEE-6FBF-4DFB-8A09-40331166CDC9}"/>
 </file>
</xml_diff>